<commit_message>
docs: corregir referencia a deploy.yml obsoleto en requisitos no funcionales
RNF-17 describia el workflow de deploy que se elimino en la Sesion 3
(integracion nativa Vercel-GitHub). Actualizado para reflejar el gateo
de migraciones por $VERCEL_ENV=production en el buildCommand de
vercel.json. Se actualiza tambien la fecha del documento.
</commit_message>
<xml_diff>
--- a/docs/REQUISITOS_INSOLVENTIC.xlsx
+++ b/docs/REQUISITOS_INSOLVENTIC.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requisitos Funcionales" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requisitos No Funcionales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Requisitos Funcionales" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Requisitos No Funcionales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requisitos Funcionales'!$A$1:$F$49</definedName>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>deploy.yml corre prisma migrate deploy antes del build, evita drift de schema entre entornos.</t>
+          <t>Migraciones gateadas por $VERCEL_ENV=production dentro del buildCommand de vercel.json; corren antes del build en cada push a main, sin workflow de CI dedicado al deploy (la integracion nativa Vercel-GitHub gestiona el build/publish).</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2814,7 +2814,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Derivado de src/features/*, README.md y las decisiones de arquitectura documentadas (ARQUITECTURA.md, CLAUDE.md). Agosto 2026.</t>
+          <t>Derivado de src/features/*, README.md y las decisiones de arquitectura documentadas (ARQUITECTURA.md, CLAUDE.md). Actualizado Octubre 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>